<commit_message>
feature(variability): worked on analysis to understand relation between kcat variation and flux rates
</commit_message>
<xml_diff>
--- a/Results/data_reduction_results/r_squared_for_analysis.xlsx
+++ b/Results/data_reduction_results/r_squared_for_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>perc_data</t>
   </si>
@@ -50,6 +50,18 @@
   </si>
   <si>
     <t>smape_EX_co2_e</t>
+  </si>
+  <si>
+    <t>pearsonr_EX_ac_e_EX_glc__D_e</t>
+  </si>
+  <si>
+    <t>pearsonr_EX_o2_e_EX_glc__D_e</t>
+  </si>
+  <si>
+    <t>pearsonr_BIOMASS_Ec_iML1515_core_75p37M_EX_glc__D_e</t>
+  </si>
+  <si>
+    <t>pearsonr_EX_co2_e_EX_glc__D_e</t>
   </si>
 </sst>
 </file>
@@ -407,10 +419,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,8 +459,20 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
       <c r="A2">
         <v>10</v>
       </c>
@@ -456,37 +480,49 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>0.4478640163516427</v>
+        <v>0.4478640947623611</v>
       </c>
       <c r="D2">
-        <v>0.2620557831284377</v>
+        <v>0.2620557832923219</v>
       </c>
       <c r="E2">
-        <v>0.8585080860547227</v>
+        <v>0.8585080861030872</v>
       </c>
       <c r="F2">
-        <v>0.7944975367920385</v>
+        <v>0.7944978500748618</v>
       </c>
       <c r="G2">
-        <v>-0.1236053405686282</v>
+        <v>-0.1236053404208266</v>
       </c>
       <c r="H2">
-        <v>83.66715072827631</v>
+        <v>83.66712740782647</v>
       </c>
       <c r="I2">
-        <v>57.25102470206098</v>
+        <v>57.25102470020842</v>
       </c>
       <c r="J2">
-        <v>141.4853743464418</v>
+        <v>141.485374336236</v>
       </c>
       <c r="K2">
-        <v>18.66176702612878</v>
+        <v>18.66167376565772</v>
       </c>
       <c r="L2">
-        <v>117.2704368384736</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>117.2704368292037</v>
+      </c>
+      <c r="M2">
+        <v>0.9360539969456827</v>
+      </c>
+      <c r="N2">
+        <v>0.9430611895432159</v>
+      </c>
+      <c r="O2">
+        <v>0.9697306421537695</v>
+      </c>
+      <c r="P2">
+        <v>0.79671823732509</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
       <c r="A3">
         <v>10</v>
       </c>
@@ -494,37 +530,49 @@
         <v>6</v>
       </c>
       <c r="C3">
-        <v>-0.03931091276063114</v>
+        <v>-0.03934163857506345</v>
       </c>
       <c r="D3">
-        <v>0.3284698053512283</v>
+        <v>0.328469805398245</v>
       </c>
       <c r="E3">
-        <v>0.2577771759149633</v>
+        <v>0.2577506596884387</v>
       </c>
       <c r="F3">
-        <v>0.7210269583085939</v>
+        <v>0.7210197635180009</v>
       </c>
       <c r="G3">
-        <v>-1.46451759061731</v>
+        <v>-1.464606782904939</v>
       </c>
       <c r="H3">
-        <v>86.12550863599984</v>
+        <v>86.12595861804712</v>
       </c>
       <c r="I3">
-        <v>56.4882153215805</v>
+        <v>56.48821532401755</v>
       </c>
       <c r="J3">
-        <v>143.41100363564</v>
+        <v>143.411292279557</v>
       </c>
       <c r="K3">
-        <v>23.6186676972408</v>
+        <v>23.61958573809026</v>
       </c>
       <c r="L3">
-        <v>120.984147889538</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>120.9847411305237</v>
+      </c>
+      <c r="M3">
+        <v>0.7269753958866909</v>
+      </c>
+      <c r="N3">
+        <v>0.8093116949510788</v>
+      </c>
+      <c r="O3">
+        <v>0.9698688737903991</v>
+      </c>
+      <c r="P3">
+        <v>0.6162377363297997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
       <c r="A4">
         <v>10</v>
       </c>
@@ -532,37 +580,49 @@
         <v>7</v>
       </c>
       <c r="C4">
-        <v>0.002888910716147108</v>
+        <v>0.002868426848591121</v>
       </c>
       <c r="D4">
-        <v>0.3586490432652814</v>
+        <v>0.3586490432769955</v>
       </c>
       <c r="E4">
-        <v>0.2365757415820797</v>
+        <v>0.2365580641062378</v>
       </c>
       <c r="F4">
-        <v>0.7719247461080663</v>
+        <v>0.7719199495781226</v>
       </c>
       <c r="G4">
-        <v>-1.355593888090839</v>
+        <v>-1.355653349566992</v>
       </c>
       <c r="H4">
-        <v>85.13829298727526</v>
+        <v>85.13859297715578</v>
       </c>
       <c r="I4">
-        <v>55.66994664016613</v>
+        <v>55.66994664315638</v>
       </c>
       <c r="J4">
-        <v>143.3785131925617</v>
+        <v>143.3787056192628</v>
       </c>
       <c r="K4">
-        <v>21.22217697728806</v>
+        <v>21.22278901550156</v>
       </c>
       <c r="L4">
-        <v>120.2825351390851</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>120.2829306307023</v>
+      </c>
+      <c r="M4">
+        <v>0.7245646483567534</v>
+      </c>
+      <c r="N4">
+        <v>0.8267837922565925</v>
+      </c>
+      <c r="O4">
+        <v>0.9753486884822957</v>
+      </c>
+      <c r="P4">
+        <v>0.6128987796139895</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
       <c r="A5">
         <v>10</v>
       </c>
@@ -570,37 +630,49 @@
         <v>8</v>
       </c>
       <c r="C5">
-        <v>-0.0001831176337696583</v>
+        <v>-0.06430538208514366</v>
       </c>
       <c r="D5">
-        <v>0.2085724134811284</v>
+        <v>-0.4391578084185936</v>
       </c>
       <c r="E5">
-        <v>0.2674986679988738</v>
+        <v>0.3910235185556307</v>
       </c>
       <c r="F5">
-        <v>0.5304337726039706</v>
+        <v>0.6899610687051254</v>
       </c>
       <c r="G5">
-        <v>-1.007237324619052</v>
+        <v>-0.8990483071827371</v>
       </c>
       <c r="H5">
-        <v>89.8439987601999</v>
+        <v>86.99693950945918</v>
       </c>
       <c r="I5">
-        <v>67.52912070561339</v>
+        <v>62.36122766965651</v>
       </c>
       <c r="J5">
-        <v>143.9301153794046</v>
+        <v>142.9017094669051</v>
       </c>
       <c r="K5">
-        <v>28.32458922666637</v>
+        <v>23.57053783079896</v>
       </c>
       <c r="L5">
-        <v>119.5921697291152</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>119.1542830704761</v>
+      </c>
+      <c r="M5">
+        <v>0.7245646483567534</v>
+      </c>
+      <c r="N5">
+        <v>0.8325009329522249</v>
+      </c>
+      <c r="O5">
+        <v>0.9821805230861609</v>
+      </c>
+      <c r="P5">
+        <v>0.6210005087035206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6">
         <v>20</v>
       </c>
@@ -608,37 +680,49 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>0.09682961856171335</v>
+        <v>0.04553132377047736</v>
       </c>
       <c r="D6">
-        <v>0.2427678182864965</v>
+        <v>-0.275416359208045</v>
       </c>
       <c r="E6">
-        <v>0.3860163418212236</v>
+        <v>0.484835218791924</v>
       </c>
       <c r="F6">
-        <v>0.5910629823342908</v>
+        <v>0.7186847491686448</v>
       </c>
       <c r="G6">
-        <v>-0.8325286681951574</v>
+        <v>-0.7459783136706144</v>
       </c>
       <c r="H6">
-        <v>88.49581099491144</v>
+        <v>86.21818165592687</v>
       </c>
       <c r="I6">
-        <v>65.14720128431321</v>
+        <v>61.01288685542088</v>
       </c>
       <c r="J6">
-        <v>143.3930098178411</v>
+        <v>142.570334813454</v>
       </c>
       <c r="K6">
-        <v>26.25244417838948</v>
+        <v>22.44918105065833</v>
       </c>
       <c r="L6">
-        <v>119.1905886991019</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>118.8403239041743</v>
+      </c>
+      <c r="M6">
+        <v>0.7020928195336119</v>
+      </c>
+      <c r="N6">
+        <v>0.7970813463158941</v>
+      </c>
+      <c r="O6">
+        <v>0.9742713006977861</v>
+      </c>
+      <c r="P6">
+        <v>0.6225097430182274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
       <c r="A7">
         <v>20</v>
       </c>
@@ -646,37 +730,49 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>-0.241098016493056</v>
+        <v>-0.2094824127082397</v>
       </c>
       <c r="D7">
-        <v>-0.3306048230667502</v>
+        <v>-0.7879343187380046</v>
       </c>
       <c r="E7">
-        <v>0.1224451392624798</v>
+        <v>0.34186585383171</v>
       </c>
       <c r="F7">
-        <v>0.1537724872492702</v>
+        <v>0.3001185141336602</v>
       </c>
       <c r="G7">
-        <v>-0.9100048694172236</v>
+        <v>-0.6919797000603243</v>
       </c>
       <c r="H7">
-        <v>99.04814371844506</v>
+        <v>95.53215602355203</v>
       </c>
       <c r="I7">
-        <v>80.77757937052455</v>
+        <v>75.47871017513415</v>
       </c>
       <c r="J7">
-        <v>146.1149806081022</v>
+        <v>144.5909148764264</v>
       </c>
       <c r="K7">
-        <v>47.63585526353544</v>
+        <v>42.15910280382179</v>
       </c>
       <c r="L7">
-        <v>121.664159631618</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>119.8998962388258</v>
+      </c>
+      <c r="M7">
+        <v>0.9144757523768708</v>
+      </c>
+      <c r="N7">
+        <v>0.9079239833375148</v>
+      </c>
+      <c r="O7">
+        <v>0.8550706011930316</v>
+      </c>
+      <c r="P7">
+        <v>0.8497272875509576</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
       <c r="A8">
         <v>20</v>
       </c>
@@ -684,37 +780,49 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>-0.3840608302227648</v>
+        <v>-0.5067965755035844</v>
       </c>
       <c r="D8">
-        <v>-0.3374811045800388</v>
+        <v>-1.66609423692069</v>
       </c>
       <c r="E8">
-        <v>0.0364141522068836</v>
+        <v>0.3227765942094396</v>
       </c>
       <c r="F8">
-        <v>-0.2066513087997388</v>
+        <v>-0.07923617678711459</v>
       </c>
       <c r="G8">
-        <v>-1.028525059718165</v>
+        <v>-0.6046324825159719</v>
       </c>
       <c r="H8">
-        <v>108.8708349723155</v>
+        <v>104.3467070237614</v>
       </c>
       <c r="I8">
-        <v>95.01005110290942</v>
+        <v>87.80645400061402</v>
       </c>
       <c r="J8">
-        <v>147.2949302821688</v>
+        <v>145.4021990420032</v>
       </c>
       <c r="K8">
-        <v>69.12969994472661</v>
+        <v>64.31844769076473</v>
       </c>
       <c r="L8">
-        <v>124.0486585594574</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>119.8597273616635</v>
+      </c>
+      <c r="M8">
+        <v>0.9458755153182261</v>
+      </c>
+      <c r="N8">
+        <v>0.8528931086322128</v>
+      </c>
+      <c r="O8">
+        <v>0.7311775221960557</v>
+      </c>
+      <c r="P8">
+        <v>0.828746218678051</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
       <c r="A9">
         <v>20</v>
       </c>
@@ -722,37 +830,49 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>-0.2822659095237713</v>
+        <v>-0.3896630917746426</v>
       </c>
       <c r="D9">
-        <v>-0.2242484397332363</v>
+        <v>-1.386784930528945</v>
       </c>
       <c r="E9">
-        <v>0.1271719665999468</v>
+        <v>0.3777379325363077</v>
       </c>
       <c r="F9">
-        <v>-0.06934256993751675</v>
+        <v>0.04214531176169301</v>
       </c>
       <c r="G9">
-        <v>-0.9626445950242788</v>
+        <v>-0.5917506808676267</v>
       </c>
       <c r="H9">
-        <v>105.3792076980351</v>
+        <v>101.4206236757103</v>
       </c>
       <c r="I9">
-        <v>89.04077839045918</v>
+        <v>82.73763092652285</v>
       </c>
       <c r="J9">
-        <v>146.5971346350991</v>
+        <v>144.9409989605669</v>
       </c>
       <c r="K9">
-        <v>62.47490472143674</v>
+        <v>58.26506552624329</v>
       </c>
       <c r="L9">
-        <v>123.4040130451456</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>119.7387992895083</v>
+      </c>
+      <c r="M9">
+        <v>0.9528230592221227</v>
+      </c>
+      <c r="N9">
+        <v>0.860033873163482</v>
+      </c>
+      <c r="O9">
+        <v>0.690262958229295</v>
+      </c>
+      <c r="P9">
+        <v>0.7858405999270188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
       <c r="A10">
         <v>30</v>
       </c>
@@ -760,37 +880,49 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>-0.4958088136817542</v>
+        <v>-0.6170705250253017</v>
       </c>
       <c r="D10">
-        <v>-0.4566798844022528</v>
+        <v>-2.098651083654998</v>
       </c>
       <c r="E10">
-        <v>-0.02116809262511121</v>
+        <v>0.367731966513846</v>
       </c>
       <c r="F10">
-        <v>-0.3204328390468725</v>
+        <v>-0.2175100955764295</v>
       </c>
       <c r="G10">
-        <v>-1.18495443865278</v>
+        <v>-0.519852887383625</v>
       </c>
       <c r="H10">
-        <v>113.1234530040833</v>
+        <v>107.4795657833575</v>
       </c>
       <c r="I10">
-        <v>100.7085129794976</v>
+        <v>92.21007172528883</v>
       </c>
       <c r="J10">
-        <v>148.0943364801248</v>
+        <v>145.3758555019476</v>
       </c>
       <c r="K10">
-        <v>76.86170686841513</v>
+        <v>72.88927644995823</v>
       </c>
       <c r="L10">
-        <v>126.8292556882955</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>119.4430594562351</v>
+      </c>
+      <c r="M10">
+        <v>0.8494891483170348</v>
+      </c>
+      <c r="N10">
+        <v>0.8203151999681275</v>
+      </c>
+      <c r="O10">
+        <v>0.7651952951137077</v>
+      </c>
+      <c r="P10">
+        <v>0.7399077426616307</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
       <c r="A11">
         <v>30</v>
       </c>
@@ -798,37 +930,49 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>-0.4234825139129409</v>
+        <v>-0.5326178922384162</v>
       </c>
       <c r="D11">
-        <v>-0.4048709279026275</v>
+        <v>-1.882645007244373</v>
       </c>
       <c r="E11">
-        <v>0.02638276505324566</v>
+        <v>0.3763925547927823</v>
       </c>
       <c r="F11">
-        <v>-0.191702824247721</v>
+        <v>-0.09907236090801375</v>
       </c>
       <c r="G11">
-        <v>-1.123739068554661</v>
+        <v>-0.5251467555940605</v>
       </c>
       <c r="H11">
-        <v>110.3768568527404</v>
+        <v>105.2973532949912</v>
       </c>
       <c r="I11">
-        <v>97.45015664725175</v>
+        <v>89.80155951888666</v>
       </c>
       <c r="J11">
-        <v>147.5905140129657</v>
+        <v>145.1438888663613</v>
       </c>
       <c r="K11">
-        <v>70.57317219553084</v>
+        <v>66.99798382388232</v>
       </c>
       <c r="L11">
-        <v>125.8935845552133</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <v>119.2459809708346</v>
+      </c>
+      <c r="M11">
+        <v>0.7121277450872898</v>
+      </c>
+      <c r="N11">
+        <v>0.9411645589427198</v>
+      </c>
+      <c r="O11">
+        <v>0.820479035757099</v>
+      </c>
+      <c r="P11">
+        <v>0.8063840550567232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
       <c r="A12">
         <v>30</v>
       </c>
@@ -836,37 +980,49 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>-0.5620720158991207</v>
+        <v>-0.6613982832653059</v>
       </c>
       <c r="D12">
-        <v>-0.3968084121803164</v>
+        <v>-1.740076454240136</v>
       </c>
       <c r="E12">
-        <v>-0.1104512537137965</v>
+        <v>0.2322579234867128</v>
       </c>
       <c r="F12">
-        <v>-0.3880604422421052</v>
+        <v>-0.3004817620212801</v>
       </c>
       <c r="G12">
-        <v>-1.352967955460265</v>
+        <v>-0.8372928402865201</v>
       </c>
       <c r="H12">
-        <v>116.9841090269919</v>
+        <v>112.3454430520664</v>
       </c>
       <c r="I12">
-        <v>106.750711093889</v>
+        <v>99.7678998267973</v>
       </c>
       <c r="J12">
-        <v>149.0238256076018</v>
+        <v>146.6497868629739</v>
       </c>
       <c r="K12">
-        <v>81.91215972013605</v>
+        <v>78.32896687865176</v>
       </c>
       <c r="L12">
-        <v>130.2497396863409</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <v>124.6351186398425</v>
+      </c>
+      <c r="M12">
+        <v>0.7704676343311261</v>
+      </c>
+      <c r="N12">
+        <v>0.7732247974313264</v>
+      </c>
+      <c r="O12">
+        <v>0.8282647631068217</v>
+      </c>
+      <c r="P12">
+        <v>0.7292244360939615</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
       <c r="A13">
         <v>30</v>
       </c>
@@ -874,37 +1030,49 @@
         <v>8</v>
       </c>
       <c r="C13">
-        <v>-0.5472080301605018</v>
+        <v>-0.6382571085568001</v>
       </c>
       <c r="D13">
-        <v>-0.6544984366652586</v>
+        <v>-1.885827475146015</v>
       </c>
       <c r="E13">
-        <v>-0.05207928586291</v>
+        <v>0.262070793243719</v>
       </c>
       <c r="F13">
-        <v>-0.2976860275094526</v>
+        <v>-0.2174055706345723</v>
       </c>
       <c r="G13">
-        <v>-1.184568370604386</v>
+        <v>-0.711866181690332</v>
       </c>
       <c r="H13">
-        <v>114.6791268369999</v>
+        <v>110.4270163597758</v>
       </c>
       <c r="I13">
-        <v>104.3807667096512</v>
+        <v>97.97985638087815</v>
       </c>
       <c r="J13">
-        <v>148.6390927908553</v>
+        <v>146.4628906082378</v>
       </c>
       <c r="K13">
-        <v>76.93991107517603</v>
+        <v>73.65531763698165</v>
       </c>
       <c r="L13">
-        <v>128.7567367723173</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>123.6100008130058</v>
+      </c>
+      <c r="M13">
+        <v>0.7280171735871246</v>
+      </c>
+      <c r="N13">
+        <v>0.8682285546326056</v>
+      </c>
+      <c r="O13">
+        <v>0.9631782044472887</v>
+      </c>
+      <c r="P13">
+        <v>0.6690558696654706</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
       <c r="A14">
         <v>40</v>
       </c>
@@ -912,37 +1080,49 @@
         <v>5</v>
       </c>
       <c r="C14">
-        <v>-0.4592788818241251</v>
+        <v>-0.5433241849480377</v>
       </c>
       <c r="D14">
-        <v>-0.5948555471180619</v>
+        <v>-1.731466967241287</v>
       </c>
       <c r="E14">
-        <v>0.01604602715049608</v>
+        <v>0.3060307155715697</v>
       </c>
       <c r="F14">
-        <v>-0.2082477275311829</v>
+        <v>-0.134142690416533</v>
       </c>
       <c r="G14">
-        <v>-1.050058279797752</v>
+        <v>-0.613717797705901</v>
       </c>
       <c r="H14">
-        <v>112.0911725224485</v>
+        <v>108.1661474656023</v>
       </c>
       <c r="I14">
-        <v>100.2073346813308</v>
+        <v>94.29880206994603</v>
       </c>
       <c r="J14">
-        <v>148.1585762146139</v>
+        <v>146.1497741971469</v>
       </c>
       <c r="K14">
-        <v>72.36270487308211</v>
+        <v>69.33077247021477</v>
       </c>
       <c r="L14">
-        <v>127.6360743207672</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <v>122.8852411251016</v>
+      </c>
+      <c r="M14">
+        <v>0.4248013217620453</v>
+      </c>
+      <c r="N14">
+        <v>0.6245424919359261</v>
+      </c>
+      <c r="O14">
+        <v>0.7133890023138847</v>
+      </c>
+      <c r="P14">
+        <v>0.5516921872393474</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
       <c r="A15">
         <v>40</v>
       </c>
@@ -950,37 +1130,49 @@
         <v>6</v>
       </c>
       <c r="C15">
-        <v>-0.4098065147602247</v>
+        <v>-0.487848581940186</v>
       </c>
       <c r="D15">
-        <v>-0.5549678514300904</v>
+        <v>-1.610392741550424</v>
       </c>
       <c r="E15">
-        <v>0.04412763569192013</v>
+        <v>0.3133991320955126</v>
       </c>
       <c r="F15">
-        <v>-0.1247431017562455</v>
+        <v>-0.05593128158585547</v>
       </c>
       <c r="G15">
-        <v>-1.003642741546483</v>
+        <v>-0.5984694367199772</v>
       </c>
       <c r="H15">
-        <v>110.2481361157628</v>
+        <v>106.6034699917858</v>
       </c>
       <c r="I15">
-        <v>98.07241064215418</v>
+        <v>92.5859160744974</v>
       </c>
       <c r="J15">
-        <v>147.8117455650358</v>
+        <v>145.9464294043978</v>
       </c>
       <c r="K15">
-        <v>68.25313531460411</v>
+        <v>65.437769515786</v>
       </c>
       <c r="L15">
-        <v>126.8552529412572</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+        <v>122.4437649724621</v>
+      </c>
+      <c r="M15">
+        <v>0.5599660591878678</v>
+      </c>
+      <c r="N15">
+        <v>0.6675746682107038</v>
+      </c>
+      <c r="O15">
+        <v>0.8050403296529087</v>
+      </c>
+      <c r="P15">
+        <v>0.5979363895570905</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
       <c r="A16">
         <v>40</v>
       </c>
@@ -988,37 +1180,49 @@
         <v>7</v>
       </c>
       <c r="C16">
-        <v>-0.344302751777182</v>
+        <v>-0.4171420144711941</v>
       </c>
       <c r="D16">
-        <v>-0.5197379242980775</v>
+        <v>-1.504801155061151</v>
       </c>
       <c r="E16">
-        <v>0.1005134632079661</v>
+        <v>0.3518335265249407</v>
       </c>
       <c r="F16">
-        <v>-0.0561416085923192</v>
+        <v>0.008082756900067212</v>
       </c>
       <c r="G16">
-        <v>-0.9018449374262973</v>
+        <v>-0.5236831862486337</v>
       </c>
       <c r="H16">
-        <v>108.4165364138239</v>
+        <v>105.0148480310076</v>
       </c>
       <c r="I16">
-        <v>95.40939927077342</v>
+        <v>90.28867100760696</v>
       </c>
       <c r="J16">
-        <v>147.3980326227223</v>
+        <v>145.6570708714707</v>
       </c>
       <c r="K16">
-        <v>64.8189541741811</v>
+        <v>62.19127942938887</v>
       </c>
       <c r="L16">
-        <v>126.0397595876189</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>121.9223708155639</v>
+      </c>
+      <c r="M16">
+        <v>0.7600473124118072</v>
+      </c>
+      <c r="N16">
+        <v>0.8942029928414117</v>
+      </c>
+      <c r="O16">
+        <v>0.808564773499898</v>
+      </c>
+      <c r="P16">
+        <v>0.8845328140147093</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16">
       <c r="A17">
         <v>40</v>
       </c>
@@ -1026,37 +1230,49 @@
         <v>8</v>
       </c>
       <c r="C17">
-        <v>-0.281166962459382</v>
+        <v>-0.3494539686610175</v>
       </c>
       <c r="D17">
-        <v>-0.4564301495900895</v>
+        <v>-1.379926928422998</v>
       </c>
       <c r="E17">
-        <v>0.1481312037222959</v>
+        <v>0.3837439166042478</v>
       </c>
       <c r="F17">
-        <v>0.006202923240095304</v>
+        <v>0.06641339913397171</v>
       </c>
       <c r="G17">
-        <v>-0.8225718272098297</v>
+        <v>-0.4680462619592913</v>
       </c>
       <c r="H17">
-        <v>106.5179096910758</v>
+        <v>103.3288256365425</v>
       </c>
       <c r="I17">
-        <v>91.90086748355263</v>
+        <v>87.10018473706262</v>
       </c>
       <c r="J17">
-        <v>147.0594724350785</v>
+        <v>145.4273205560669</v>
       </c>
       <c r="K17">
-        <v>61.74808566677906</v>
+        <v>59.28462540222335</v>
       </c>
       <c r="L17">
-        <v>125.3632131788932</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+        <v>121.5031718508171</v>
+      </c>
+      <c r="M17">
+        <v>0.8378412360046876</v>
+      </c>
+      <c r="N17">
+        <v>0.9053224547016656</v>
+      </c>
+      <c r="O17">
+        <v>0.9435091182862656</v>
+      </c>
+      <c r="P17">
+        <v>0.7623398961692458</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
       <c r="A18">
         <v>50</v>
       </c>
@@ -1064,37 +1280,49 @@
         <v>5</v>
       </c>
       <c r="C18">
-        <v>-0.2350466666086049</v>
+        <v>-0.2993167900881794</v>
       </c>
       <c r="D18">
-        <v>-0.4502050692064548</v>
+        <v>-1.319378508090006</v>
       </c>
       <c r="E18">
-        <v>0.1900425564605414</v>
+        <v>0.4117956979973202</v>
       </c>
       <c r="F18">
-        <v>0.05823842413499669</v>
+        <v>0.1149071073300699</v>
       </c>
       <c r="G18">
-        <v>-0.7382625778235028</v>
+        <v>-0.4045914575901013</v>
       </c>
       <c r="H18">
-        <v>105.0941253179095</v>
+        <v>102.0926344430764</v>
       </c>
       <c r="I18">
-        <v>89.78240815772405</v>
+        <v>85.26411851407164</v>
       </c>
       <c r="J18">
-        <v>146.7644488153325</v>
+        <v>145.2283058703643</v>
       </c>
       <c r="K18">
-        <v>59.12455463148554</v>
+        <v>56.80600379424131</v>
       </c>
       <c r="L18">
-        <v>124.7050896670961</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+        <v>121.0721095936284</v>
+      </c>
+      <c r="M18">
+        <v>0.5932043578021406</v>
+      </c>
+      <c r="N18">
+        <v>0.8096457075464536</v>
+      </c>
+      <c r="O18">
+        <v>0.8908611144790463</v>
+      </c>
+      <c r="P18">
+        <v>0.6835591558242982</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
       <c r="A19">
         <v>50</v>
       </c>
@@ -1102,37 +1330,49 @@
         <v>6</v>
       </c>
       <c r="C19">
-        <v>-0.3118060579433909</v>
+        <v>-0.3636477728273687</v>
       </c>
       <c r="D19">
-        <v>-0.5775484215670319</v>
+        <v>-1.550251566770266</v>
       </c>
       <c r="E19">
-        <v>0.1162514815144339</v>
+        <v>0.3926513690758135</v>
       </c>
       <c r="F19">
-        <v>-0.02885995545918729</v>
+        <v>0.07119826362968962</v>
       </c>
       <c r="G19">
-        <v>-0.7570673362617781</v>
+        <v>-0.3681891572447122</v>
       </c>
       <c r="H19">
-        <v>107.2585563564841</v>
+        <v>103.1239920698263</v>
       </c>
       <c r="I19">
-        <v>94.56822039011078</v>
+        <v>88.55110982975647</v>
       </c>
       <c r="J19">
-        <v>147.4139963609631</v>
+        <v>145.4659291828809</v>
       </c>
       <c r="K19">
-        <v>61.95654996249361</v>
+        <v>57.66681628528387</v>
       </c>
       <c r="L19">
-        <v>125.0954587123689</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <v>120.8121129813838</v>
+      </c>
+      <c r="M19">
+        <v>0.7558863022775006</v>
+      </c>
+      <c r="N19">
+        <v>0.9435527330736324</v>
+      </c>
+      <c r="O19">
+        <v>0.8672588670403377</v>
+      </c>
+      <c r="P19">
+        <v>0.8720901330748427</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16">
       <c r="A20">
         <v>50</v>
       </c>
@@ -1140,37 +1380,49 @@
         <v>7</v>
       </c>
       <c r="C20">
-        <v>-0.3007253994707684</v>
+        <v>-0.3498386915013973</v>
       </c>
       <c r="D20">
-        <v>-0.5589022151943326</v>
+        <v>-1.480410458018385</v>
       </c>
       <c r="E20">
-        <v>0.1058221954793186</v>
+        <v>0.3676743615372832</v>
       </c>
       <c r="F20">
-        <v>0.02323690687935698</v>
+        <v>0.118028821522717</v>
       </c>
       <c r="G20">
-        <v>-0.7730584850474167</v>
+        <v>-0.404647491047204</v>
       </c>
       <c r="H20">
-        <v>106.1718244850543</v>
+        <v>102.2548734718613</v>
       </c>
       <c r="I20">
-        <v>93.31035583026768</v>
+        <v>87.6099352994041</v>
       </c>
       <c r="J20">
-        <v>147.2135261068615</v>
+        <v>145.3679964098159</v>
       </c>
       <c r="K20">
-        <v>59.46249246944467</v>
+        <v>55.39854621842786</v>
       </c>
       <c r="L20">
-        <v>124.7009235336434</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+        <v>120.6430159597974</v>
+      </c>
+      <c r="M20">
+        <v>0.9116704448943919</v>
+      </c>
+      <c r="N20">
+        <v>0.7604369075840653</v>
+      </c>
+      <c r="O20">
+        <v>0.785568523197766</v>
+      </c>
+      <c r="P20">
+        <v>0.7421241555954824</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16">
       <c r="A21">
         <v>50</v>
       </c>
@@ -1178,37 +1430,49 @@
         <v>8</v>
       </c>
       <c r="C21">
-        <v>-0.2561743146076809</v>
+        <v>-0.3098259844003757</v>
       </c>
       <c r="D21">
-        <v>-0.509191673618544</v>
+        <v>-1.423381186926511</v>
       </c>
       <c r="E21">
-        <v>0.1368329724682092</v>
+        <v>0.3901011650113339</v>
       </c>
       <c r="F21">
-        <v>0.05883548354535884</v>
+        <v>0.1512058133667505</v>
       </c>
       <c r="G21">
-        <v>-0.7111740408257476</v>
+        <v>-0.3572297290530762</v>
       </c>
       <c r="H21">
-        <v>104.9577031511547</v>
+        <v>101.2790878543422</v>
       </c>
       <c r="I21">
-        <v>91.12258695923074</v>
+        <v>85.97060697774407</v>
       </c>
       <c r="J21">
-        <v>147.0096912696797</v>
+        <v>145.2242688361597</v>
       </c>
       <c r="K21">
-        <v>57.48721468097507</v>
+        <v>53.59254609051614</v>
       </c>
       <c r="L21">
-        <v>124.2113196947332</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+        <v>120.3289295129489</v>
+      </c>
+      <c r="M21">
+        <v>0.8809235107597109</v>
+      </c>
+      <c r="N21">
+        <v>0.8755846634271371</v>
+      </c>
+      <c r="O21">
+        <v>0.5575167458140067</v>
+      </c>
+      <c r="P21">
+        <v>0.806086003748929</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16">
       <c r="A22">
         <v>60</v>
       </c>
@@ -1216,37 +1480,49 @@
         <v>5</v>
       </c>
       <c r="C22">
-        <v>-0.2323267802693688</v>
+        <v>-0.2834236086620269</v>
       </c>
       <c r="D22">
-        <v>-0.5437784911894483</v>
+        <v>-1.414435170519925</v>
       </c>
       <c r="E22">
-        <v>0.167101818267204</v>
+        <v>0.4083096207192509</v>
       </c>
       <c r="F22">
-        <v>0.09305342101756886</v>
+        <v>0.1810251637059755</v>
       </c>
       <c r="G22">
-        <v>-0.6456838691727997</v>
+        <v>-0.3085940485534084</v>
       </c>
       <c r="H22">
-        <v>103.9880969546154</v>
+        <v>100.4846538155485</v>
       </c>
       <c r="I22">
-        <v>89.78651355955404</v>
+        <v>84.87986595807256</v>
       </c>
       <c r="J22">
-        <v>146.7846646251363</v>
+        <v>145.0842623066333</v>
       </c>
       <c r="K22">
-        <v>55.71183716807951</v>
+        <v>52.00262898714227</v>
       </c>
       <c r="L22">
-        <v>123.6693724656919</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
+        <v>119.971858010346</v>
+      </c>
+      <c r="M22">
+        <v>0.9746422630396467</v>
+      </c>
+      <c r="N22">
+        <v>0.9500316050562099</v>
+      </c>
+      <c r="O22">
+        <v>0.6325437062857653</v>
+      </c>
+      <c r="P22">
+        <v>0.8655092564079637</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16">
       <c r="A23">
         <v>60</v>
       </c>
@@ -1254,37 +1530,49 @@
         <v>6</v>
       </c>
       <c r="C23">
-        <v>-0.2119428605438697</v>
+        <v>-0.2607171058244228</v>
       </c>
       <c r="D23">
-        <v>-0.5843606591272927</v>
+        <v>-1.41544203483898</v>
       </c>
       <c r="E23">
-        <v>0.1941033044059406</v>
+        <v>0.424347115838392</v>
       </c>
       <c r="F23">
-        <v>0.126661077586632</v>
+        <v>0.2106341046990517</v>
       </c>
       <c r="G23">
-        <v>-0.5841751650407587</v>
+        <v>-0.2624076089961551</v>
       </c>
       <c r="H23">
-        <v>103.2487915969887</v>
+        <v>99.90459587338823</v>
       </c>
       <c r="I23">
-        <v>89.18016115665615</v>
+        <v>84.49654299183439</v>
       </c>
       <c r="J23">
-        <v>146.6143543372409</v>
+        <v>144.9912430332097</v>
       </c>
       <c r="K23">
-        <v>54.01855643100849</v>
+        <v>50.47794862190455</v>
       </c>
       <c r="L23">
-        <v>123.1820944630493</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+        <v>119.6526488466042</v>
+      </c>
+      <c r="M23">
+        <v>0.9664243281959813</v>
+      </c>
+      <c r="N23">
+        <v>0.9666728559373365</v>
+      </c>
+      <c r="O23">
+        <v>0.9191831342972047</v>
+      </c>
+      <c r="P23">
+        <v>0.8862039632129792</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16">
       <c r="A24">
         <v>60</v>
       </c>
@@ -1292,37 +1580,49 @@
         <v>7</v>
       </c>
       <c r="C24">
-        <v>-0.1815074535580707</v>
+        <v>-0.2281610794764159</v>
       </c>
       <c r="D24">
-        <v>-0.5757408481554971</v>
+        <v>-1.370688251001054</v>
       </c>
       <c r="E24">
-        <v>0.2236954526418693</v>
+        <v>0.443928663577649</v>
       </c>
       <c r="F24">
-        <v>0.1595811753321607</v>
+        <v>0.2399032012664462</v>
       </c>
       <c r="G24">
-        <v>-0.5335655940508155</v>
+        <v>-0.2257879317487046</v>
       </c>
       <c r="H24">
-        <v>102.3211321046675</v>
+        <v>99.12233619516546</v>
       </c>
       <c r="I24">
-        <v>87.65796726998096</v>
+        <v>83.17798467766292</v>
       </c>
       <c r="J24">
-        <v>146.4043877091319</v>
+        <v>144.8518464617959</v>
       </c>
       <c r="K24">
-        <v>52.42597887715029</v>
+        <v>49.03931053799608</v>
       </c>
       <c r="L24">
-        <v>122.7961945624069</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+        <v>119.4202031032069</v>
+      </c>
+      <c r="M24">
+        <v>0.8024731580997161</v>
+      </c>
+      <c r="N24">
+        <v>0.8663907617210669</v>
+      </c>
+      <c r="O24">
+        <v>0.8406960286864873</v>
+      </c>
+      <c r="P24">
+        <v>0.835600010634457</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16">
       <c r="A25">
         <v>60</v>
       </c>
@@ -1330,37 +1630,49 @@
         <v>8</v>
       </c>
       <c r="C25">
-        <v>-0.1587526782404952</v>
+        <v>-0.2034624030685528</v>
       </c>
       <c r="D25">
-        <v>-0.586853218729009</v>
+        <v>-1.348677813111185</v>
       </c>
       <c r="E25">
-        <v>0.2486324943552908</v>
+        <v>0.4596893215155607</v>
       </c>
       <c r="F25">
-        <v>0.186734087476339</v>
+        <v>0.2637093623251096</v>
       </c>
       <c r="G25">
-        <v>-0.4835240760646018</v>
+        <v>-0.1885704830036972</v>
       </c>
       <c r="H25">
-        <v>101.53014489405</v>
+        <v>98.46463214758313</v>
       </c>
       <c r="I25">
-        <v>86.46166164811079</v>
+        <v>82.1683449970099</v>
       </c>
       <c r="J25">
-        <v>146.2295369689201</v>
+        <v>144.7416849390513</v>
       </c>
       <c r="K25">
-        <v>51.03158223277108</v>
+        <v>47.78602507729932</v>
       </c>
       <c r="L25">
-        <v>122.3977987263981</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
+        <v>119.162473576972</v>
+      </c>
+      <c r="M25">
+        <v>0.9472852767867956</v>
+      </c>
+      <c r="N25">
+        <v>0.9690070759081999</v>
+      </c>
+      <c r="O25">
+        <v>0.9680132457580778</v>
+      </c>
+      <c r="P25">
+        <v>0.8658904825429516</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
       <c r="A26">
         <v>70</v>
       </c>
@@ -1368,37 +1680,49 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>-0.1458175853554624</v>
+        <v>-0.1887389211993288</v>
       </c>
       <c r="D26">
-        <v>-0.6289504489140703</v>
+        <v>-1.360302059510601</v>
       </c>
       <c r="E26">
-        <v>0.2718432314712578</v>
+        <v>0.4744577855580511</v>
       </c>
       <c r="F26">
-        <v>0.2103895494672795</v>
+        <v>0.2842858133216831</v>
       </c>
       <c r="G26">
-        <v>-0.4365526734463168</v>
+        <v>-0.1533972241664485</v>
       </c>
       <c r="H26">
-        <v>100.7994780943402</v>
+        <v>97.8565858582426</v>
       </c>
       <c r="I26">
-        <v>85.29656608361675</v>
+        <v>81.17498209855938</v>
       </c>
       <c r="J26">
-        <v>146.0843534380537</v>
+        <v>144.6560154882524</v>
       </c>
       <c r="K26">
-        <v>49.78172514730964</v>
+        <v>46.6659902805308</v>
       </c>
       <c r="L26">
-        <v>122.0352677083808</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+        <v>118.9293555656278</v>
+      </c>
+      <c r="M26">
+        <v>0.5810731175324965</v>
+      </c>
+      <c r="N26">
+        <v>0.7842295162900288</v>
+      </c>
+      <c r="O26">
+        <v>0.7497865256162273</v>
+      </c>
+      <c r="P26">
+        <v>0.7227194410013447</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16">
       <c r="A27">
         <v>70</v>
       </c>
@@ -1406,37 +1730,49 @@
         <v>6</v>
       </c>
       <c r="C27">
-        <v>-0.1237533152003237</v>
+        <v>-0.1650238304323083</v>
       </c>
       <c r="D27">
-        <v>-0.6285756381629206</v>
+        <v>-1.331798340649646</v>
       </c>
       <c r="E27">
-        <v>0.2928680552757658</v>
+        <v>0.4876897418984426</v>
       </c>
       <c r="F27">
-        <v>0.2358489954123134</v>
+        <v>0.3069030952729778</v>
       </c>
       <c r="G27">
-        <v>-0.3951546733264535</v>
+        <v>-0.1228898182510074</v>
       </c>
       <c r="H27">
-        <v>100.0674081438166</v>
+        <v>97.23770407063722</v>
       </c>
       <c r="I27">
-        <v>84.05554303555657</v>
+        <v>80.09248151144016</v>
       </c>
       <c r="J27">
-        <v>145.9463714979779</v>
+        <v>144.5729696231568</v>
       </c>
       <c r="K27">
-        <v>48.54519586039935</v>
+        <v>45.54929695002382</v>
       </c>
       <c r="L27">
-        <v>121.7225221813324</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
+        <v>118.7360681979281</v>
+      </c>
+      <c r="M27">
+        <v>0.981482207839225</v>
+      </c>
+      <c r="N27">
+        <v>0.9381503175350808</v>
+      </c>
+      <c r="O27">
+        <v>0.9592152776789742</v>
+      </c>
+      <c r="P27">
+        <v>0.9163148339301477</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16">
       <c r="A28">
         <v>70</v>
       </c>
@@ -1444,37 +1780,49 @@
         <v>7</v>
       </c>
       <c r="C28">
-        <v>-0.1153862029221058</v>
+        <v>-0.1606125327494535</v>
       </c>
       <c r="D28">
-        <v>-0.6463882309870304</v>
+        <v>-1.361119670891261</v>
       </c>
       <c r="E28">
-        <v>0.2991138493482149</v>
+        <v>0.4944038491320729</v>
       </c>
       <c r="F28">
-        <v>0.2480353899460767</v>
+        <v>0.3197111443003026</v>
       </c>
       <c r="G28">
-        <v>-0.3623058199956846</v>
+        <v>-0.09544545353892886</v>
       </c>
       <c r="H28">
-        <v>99.66309256813963</v>
+        <v>96.9413772234048</v>
       </c>
       <c r="I28">
-        <v>83.68060857845209</v>
+        <v>79.98418167827559</v>
       </c>
       <c r="J28">
-        <v>145.9010346416383</v>
+        <v>144.5338568808957</v>
       </c>
       <c r="K28">
-        <v>47.66388421367137</v>
+        <v>44.72856453003799</v>
       </c>
       <c r="L28">
-        <v>121.4068428387967</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+        <v>118.5189058044099</v>
+      </c>
+      <c r="M28">
+        <v>0.6897638248244998</v>
+      </c>
+      <c r="N28">
+        <v>0.8397636358211027</v>
+      </c>
+      <c r="O28">
+        <v>0.9344280952781264</v>
+      </c>
+      <c r="P28">
+        <v>0.7286938079971916</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16">
       <c r="A29">
         <v>70</v>
       </c>
@@ -1482,37 +1830,49 @@
         <v>8</v>
       </c>
       <c r="C29">
-        <v>-0.09106449015383875</v>
+        <v>-0.1346755939134461</v>
       </c>
       <c r="D29">
-        <v>-0.6066856516076164</v>
+        <v>-1.295890968655192</v>
       </c>
       <c r="E29">
-        <v>0.3182695273858965</v>
+        <v>0.5065848843217908</v>
       </c>
       <c r="F29">
-        <v>0.2714638427581222</v>
+        <v>0.3405797487412627</v>
       </c>
       <c r="G29">
-        <v>-0.3473056791517573</v>
+        <v>-0.08997604006164583</v>
       </c>
       <c r="H29">
-        <v>99.1119114466735</v>
+        <v>96.4874002218173</v>
       </c>
       <c r="I29">
-        <v>82.92782759926133</v>
+        <v>79.3634159455617</v>
       </c>
       <c r="J29">
-        <v>145.7532958443478</v>
+        <v>144.434945860407</v>
       </c>
       <c r="K29">
-        <v>46.56333816859092</v>
+        <v>43.73285133316318</v>
       </c>
       <c r="L29">
-        <v>121.2031841744939</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12">
+        <v>118.4183877481373</v>
+      </c>
+      <c r="M29">
+        <v>0.5126398823602629</v>
+      </c>
+      <c r="N29">
+        <v>0.8680645009207343</v>
+      </c>
+      <c r="O29">
+        <v>0.8600404828121121</v>
+      </c>
+      <c r="P29">
+        <v>0.7498830320614942</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16">
       <c r="A30">
         <v>80</v>
       </c>
@@ -1520,37 +1880,49 @@
         <v>5</v>
       </c>
       <c r="C30">
-        <v>-0.06931750807321507</v>
+        <v>-0.1114247806610112</v>
       </c>
       <c r="D30">
-        <v>-0.5915087361366691</v>
+        <v>-1.256948352590151</v>
       </c>
       <c r="E30">
-        <v>0.3372606631393542</v>
+        <v>0.5190823870885803</v>
       </c>
       <c r="F30">
-        <v>0.2913438992267994</v>
+        <v>0.3580764981029417</v>
       </c>
       <c r="G30">
-        <v>-0.3143658585223448</v>
+        <v>-0.0659096552454157</v>
       </c>
       <c r="H30">
-        <v>98.51281068776834</v>
+        <v>95.97879985012425</v>
       </c>
       <c r="I30">
-        <v>81.89894566237345</v>
+        <v>78.45744475536728</v>
       </c>
       <c r="J30">
-        <v>145.619324680226</v>
+        <v>144.3464350395861</v>
       </c>
       <c r="K30">
-        <v>45.57673496111394</v>
+        <v>42.84385112241218</v>
       </c>
       <c r="L30">
-        <v>120.95623744736</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
+        <v>118.2674684831314</v>
+      </c>
+      <c r="M30">
+        <v>0.7490450926516721</v>
+      </c>
+      <c r="N30">
+        <v>0.9187587525892343</v>
+      </c>
+      <c r="O30">
+        <v>0.6734658737507587</v>
+      </c>
+      <c r="P30">
+        <v>0.8450911782745942</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
       <c r="A31">
         <v>80</v>
       </c>
@@ -1558,37 +1930,49 @@
         <v>6</v>
       </c>
       <c r="C31">
-        <v>-0.04589462864602561</v>
+        <v>-0.08659837376151924</v>
       </c>
       <c r="D31">
-        <v>-0.5620793024649973</v>
+        <v>-1.205337598363774</v>
       </c>
       <c r="E31">
-        <v>0.3552025653694107</v>
+        <v>0.5309636158749218</v>
       </c>
       <c r="F31">
-        <v>0.3120593086658291</v>
+        <v>0.3765675444253755</v>
       </c>
       <c r="G31">
-        <v>-0.288761086154345</v>
+        <v>-0.04858705698260013</v>
       </c>
       <c r="H31">
-        <v>97.9675201876916</v>
+        <v>95.51797612401565</v>
       </c>
       <c r="I31">
-        <v>81.01094687586678</v>
+        <v>77.68416266573932</v>
       </c>
       <c r="J31">
-        <v>145.4975786589123</v>
+        <v>144.2671197377691</v>
       </c>
       <c r="K31">
-        <v>44.60555280882372</v>
+        <v>41.96375885198368</v>
       </c>
       <c r="L31">
-        <v>120.7560024071636</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+        <v>118.1568632405704</v>
+      </c>
+      <c r="M31">
+        <v>0.9167835726060881</v>
+      </c>
+      <c r="N31">
+        <v>0.8782649886391691</v>
+      </c>
+      <c r="O31">
+        <v>0.4664895194128724</v>
+      </c>
+      <c r="P31">
+        <v>0.9085587052625301</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
       <c r="A32">
         <v>80</v>
       </c>
@@ -1596,37 +1980,49 @@
         <v>7</v>
       </c>
       <c r="C32">
-        <v>-0.09395930718845102</v>
+        <v>-0.1263632979222384</v>
       </c>
       <c r="D32">
-        <v>-0.7037900208666603</v>
+        <v>-1.309709580383584</v>
       </c>
       <c r="E32">
-        <v>0.3489598927679799</v>
+        <v>0.5223211606939012</v>
       </c>
       <c r="F32">
-        <v>0.2641095752128958</v>
+        <v>0.3269525631713698</v>
       </c>
       <c r="G32">
-        <v>-0.2851166758680195</v>
+        <v>-0.04501733517064088</v>
       </c>
       <c r="H32">
-        <v>99.01285224721782</v>
+        <v>96.53933205244569</v>
       </c>
       <c r="I32">
-        <v>83.5723205409106</v>
+        <v>79.98928833197624</v>
       </c>
       <c r="J32">
-        <v>145.5922159131423</v>
+        <v>144.3875286207155</v>
       </c>
       <c r="K32">
-        <v>46.26583238478796</v>
+        <v>43.70413289525856</v>
       </c>
       <c r="L32">
-        <v>120.6210401500304</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12">
+        <v>118.0763783618325</v>
+      </c>
+      <c r="M32">
+        <v>0.5135904611706141</v>
+      </c>
+      <c r="N32">
+        <v>0.7536342182232538</v>
+      </c>
+      <c r="O32">
+        <v>0.7913005483451229</v>
+      </c>
+      <c r="P32">
+        <v>0.5976573517478105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16">
       <c r="A33">
         <v>80</v>
       </c>
@@ -1634,37 +2030,49 @@
         <v>8</v>
       </c>
       <c r="C33">
-        <v>-0.08527238880551505</v>
+        <v>-0.1342461557543081</v>
       </c>
       <c r="D33">
-        <v>-0.7068342930552494</v>
+        <v>-1.379698327903151</v>
       </c>
       <c r="E33">
-        <v>0.3499430116562094</v>
+        <v>0.527257877968982</v>
       </c>
       <c r="F33">
-        <v>0.2711841132103624</v>
+        <v>0.3367914943468735</v>
       </c>
       <c r="G33">
-        <v>-0.2553823870333827</v>
+        <v>-0.02133566742993698</v>
       </c>
       <c r="H33">
-        <v>98.73456442231972</v>
+        <v>96.32406765275948</v>
       </c>
       <c r="I33">
-        <v>83.34598015818528</v>
+        <v>79.97458042451071</v>
       </c>
       <c r="J33">
-        <v>145.5875356913572</v>
+        <v>144.3580942683968</v>
       </c>
       <c r="K33">
-        <v>45.64286982363684</v>
+        <v>43.07853643396835</v>
       </c>
       <c r="L33">
-        <v>120.3618720160995</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+        <v>117.885059484162</v>
+      </c>
+      <c r="M33">
+        <v>0.9065351315643169</v>
+      </c>
+      <c r="N33">
+        <v>0.9068046670767207</v>
+      </c>
+      <c r="O33">
+        <v>0.8078476557085529</v>
+      </c>
+      <c r="P33">
+        <v>0.9478110054114628</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16">
       <c r="A34">
         <v>90</v>
       </c>
@@ -1672,37 +2080,49 @@
         <v>5</v>
       </c>
       <c r="C34">
-        <v>-0.06534227373779208</v>
+        <v>-0.112832040869505</v>
       </c>
       <c r="D34">
-        <v>-0.6868652165302902</v>
+        <v>-1.339339432140377</v>
       </c>
       <c r="E34">
-        <v>0.3668891219917746</v>
+        <v>0.5388306615806271</v>
       </c>
       <c r="F34">
-        <v>0.2887415598939373</v>
+        <v>0.3523607645505994</v>
       </c>
       <c r="G34">
-        <v>-0.2301345603065901</v>
+        <v>-0.003180157468869238</v>
       </c>
       <c r="H34">
-        <v>98.23751308993154</v>
+        <v>95.90006448550631</v>
       </c>
       <c r="I34">
-        <v>82.50665463021259</v>
+        <v>79.2374185248312</v>
       </c>
       <c r="J34">
-        <v>145.4602576304798</v>
+        <v>144.2680746457212</v>
       </c>
       <c r="K34">
-        <v>44.80593260029769</v>
+        <v>42.31931572859754</v>
       </c>
       <c r="L34">
-        <v>120.177207498736</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+        <v>117.7754490428753</v>
+      </c>
+      <c r="M34">
+        <v>0.8342702644188535</v>
+      </c>
+      <c r="N34">
+        <v>0.9122149508817854</v>
+      </c>
+      <c r="O34">
+        <v>0.9402131045864786</v>
+      </c>
+      <c r="P34">
+        <v>0.8182747536903601</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16">
       <c r="A35">
         <v>90</v>
       </c>
@@ -1710,37 +2130,49 @@
         <v>6</v>
       </c>
       <c r="C35">
-        <v>-0.06529340427990446</v>
+        <v>-0.1113864045348464</v>
       </c>
       <c r="D35">
-        <v>-0.6702430491701026</v>
+        <v>-1.30352684667389</v>
       </c>
       <c r="E35">
-        <v>0.3523015681993303</v>
+        <v>0.5191860669459226</v>
       </c>
       <c r="F35">
-        <v>0.3080739108370263</v>
+        <v>0.3698220005154648</v>
       </c>
       <c r="G35">
-        <v>-0.2513060469858719</v>
+        <v>-0.03102683892688307</v>
       </c>
       <c r="H35">
-        <v>97.85577084952274</v>
+        <v>95.5870701625543</v>
       </c>
       <c r="I35">
-        <v>81.97549650966384</v>
+        <v>78.8024144073768</v>
       </c>
       <c r="J35">
-        <v>145.4123697787851</v>
+        <v>144.2552512952806</v>
       </c>
       <c r="K35">
-        <v>43.94764383651476</v>
+        <v>41.53415995564779</v>
       </c>
       <c r="L35">
-        <v>120.0875732731272</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+        <v>117.756454991912</v>
+      </c>
+      <c r="M35">
+        <v>0.5317182316816944</v>
+      </c>
+      <c r="N35">
+        <v>0.7223497294636166</v>
+      </c>
+      <c r="O35">
+        <v>0.877723251473995</v>
+      </c>
+      <c r="P35">
+        <v>0.6025434625148657</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16">
       <c r="A36">
         <v>90</v>
       </c>
@@ -1748,37 +2180,49 @@
         <v>7</v>
       </c>
       <c r="C36">
-        <v>-0.05132581658359292</v>
+        <v>-0.09610187397257425</v>
       </c>
       <c r="D36">
-        <v>-0.6629618391141863</v>
+        <v>-1.278151813827884</v>
       </c>
       <c r="E36">
-        <v>0.3642557991076864</v>
+        <v>0.5263721693211963</v>
       </c>
       <c r="F36">
-        <v>0.3221577200654328</v>
+        <v>0.3821415786104553</v>
       </c>
       <c r="G36">
-        <v>-0.2287549463933045</v>
+        <v>-0.01476942999406416</v>
       </c>
       <c r="H36">
-        <v>97.53889781927705</v>
+        <v>95.33501715177471</v>
       </c>
       <c r="I36">
-        <v>81.65635645014359</v>
+        <v>78.57393383645945</v>
       </c>
       <c r="J36">
-        <v>145.33295252371</v>
+        <v>144.2088945678218</v>
       </c>
       <c r="K36">
-        <v>43.25443538101694</v>
+        <v>40.90990818261734</v>
       </c>
       <c r="L36">
-        <v>119.9118469222377</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+        <v>117.6473320202003</v>
+      </c>
+      <c r="M36">
+        <v>0.9643411734159401</v>
+      </c>
+      <c r="N36">
+        <v>0.9343750031563016</v>
+      </c>
+      <c r="O36">
+        <v>0.7798054884565532</v>
+      </c>
+      <c r="P36">
+        <v>0.918618619439739</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16">
       <c r="A37">
         <v>90</v>
       </c>
@@ -1786,34 +2230,46 @@
         <v>8</v>
       </c>
       <c r="C37">
-        <v>-0.03553864785509711</v>
+        <v>-0.07907092587000472</v>
       </c>
       <c r="D37">
-        <v>-0.6517901101684438</v>
+        <v>-1.249891474465155</v>
       </c>
       <c r="E37">
-        <v>0.3772493681364368</v>
+        <v>0.5348625058443289</v>
       </c>
       <c r="F37">
-        <v>0.3380893497111114</v>
+        <v>0.3964069899635889</v>
       </c>
       <c r="G37">
-        <v>-0.2057031990994929</v>
+        <v>0.00233827517721874</v>
       </c>
       <c r="H37">
-        <v>97.10437305486828</v>
+        <v>94.96171129480609</v>
       </c>
       <c r="I37">
-        <v>80.89213057150862</v>
+        <v>77.89533080824994</v>
       </c>
       <c r="J37">
-        <v>145.2458433903985</v>
+        <v>144.1530092666148</v>
       </c>
       <c r="K37">
-        <v>42.52714801831854</v>
+        <v>40.24774657542323</v>
       </c>
       <c r="L37">
-        <v>119.7523702392475</v>
+        <v>117.5507585289365</v>
+      </c>
+      <c r="M37">
+        <v>0.5890899633419265</v>
+      </c>
+      <c r="N37">
+        <v>0.8473886132836136</v>
+      </c>
+      <c r="O37">
+        <v>0.9086736732595442</v>
+      </c>
+      <c r="P37">
+        <v>0.7451056856505707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>